<commit_message>
Update online dating abstract
</commit_message>
<xml_diff>
--- a/projects.xlsx
+++ b/projects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naumann\Dropbox (Privat)\lennardnau.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{184FC822-DEE1-41FD-8996-64715A7CAF62}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C758FF5E-E6B6-497C-A65E-322039A6C544}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12600" windowHeight="8484" xr2:uid="{3CBB864D-7064-4EC0-B319-6895944E5474}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12600" windowHeight="8490" xr2:uid="{3CBB864D-7064-4EC0-B319-6895944E5474}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -93,9 +93,6 @@
     <t>https://osf.io/download/4aqxm/</t>
   </si>
   <si>
-    <t>Recent meta-analyses suggest that, while contact can reduce prejudice, its effects are on average small, especially in well-powered field experimental studies with delayed outcome measurement. One of the reasons why intergroup contact may fail to produce larger effect sizes is that individuals prone to avoiding outgroup contact are both less likely to benefit from and less likely to engage in such encounters. Yet, research on the drivers of intergroup avoidance is scarce. In this study, I systematically investigate patterns and drivers of intergroup avoidance in an online dating context. In partnership with large European online dating platform, I first analyze user data to examine the extent and covariates of ethnic bias in swiping behavior. Next, users will be randomly assigned to one of three brief video treatments that are delivered on the platform and designed to test three psychological mechanism that potentially drive intergroup avoidance. Behavioral data is complemented by an endline survey, including measures on intergroup contact preference, intent, and behavior.</t>
-  </si>
-  <si>
     <t>Intergroup contact and avoidance</t>
   </si>
   <si>
@@ -178,6 +175,9 @@
   </si>
   <si>
     <t>Intergroup contact and empathy education are widely believed to foster trust, tolerance and cooperation across group lines in deeply divided societies. We test these approaches independently and jointly in the context of refugee-host relations in Lebanon, where Syrian refugees comprise a quarter of the population. Our study embeds a popular existing family psycho-social support (FPSS) program targeting vulnerable youth in a field experiment, where Syrian and Lebanese youth were randomly assigned to either heterogeneous (Lebanese-Syrian) or homogeneous (Lebanese or Syrian) FPSS groups and to an empathy education or placebo curriculum focused on physical health and nutrition. We find that contact does not meaningfully change attitudes toward the outgroup, and has little effect on participation in future contact, such as attending events celebrating the outgroup's culture 1-2 months after treatment. By contrast, we find that empathy education consistently improves both affect and policy attitudes toward the outgroup, and has positive behavioral effects. We find no evidence of positive interaction effects between the two treatments. In fact, combining contact and empathy training is less effective than either treatment alone. Our study points to empathy education as a cheaper, more scalable, and potentially more effective strategy for building social cohesion in conflict settings than intergroup contact.</t>
+  </si>
+  <si>
+    <t>Recent meta-analyses suggest that, while contact can reduce prejudice, the effects are small, particularly in well-powered field experimental studies with delayed outcome measurement. One reason intergroup contact may fail to produce larger effect sizes is that those prone to avoiding outgroup contact are less likely to benefit from or engage in such encounters. However, research into the drivers of intergroup avoidance is scarce. In this study, I systematically investigate the patterns and drivers of intergroup avoidance in an online dating context. In partnership with a large European online dating platform, I first analyse user data to examine the extent  and covariates of ethnic bias in swiping behavior. Next, I conduct a large-scale field RCT in which users are randomly assigned to one of three brief video treatments. They delivered on the platform and designed to test three psychological mechanisms that potentially drive intergroup avoidance: ingroup norms, outgroup norms, and perceived group commonality. Behavioral swiping data is complemented by an endline survey including measures of intergroup contact preference, intent, and behavior.</t>
   </si>
 </sst>
 </file>
@@ -537,9 +537,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D89CD754-C723-407F-815A-E294119BEA7C}">
   <dimension ref="A1:K8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -562,7 +562,7 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I1" t="s">
         <v>18</v>
@@ -571,33 +571,33 @@
         <v>19</v>
       </c>
       <c r="K1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
         <v>23</v>
       </c>
-      <c r="B2" t="s">
-        <v>24</v>
-      </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="H2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I2" t="s">
         <v>20</v>
@@ -606,117 +606,117 @@
         <v>21</v>
       </c>
       <c r="K2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3" t="s">
+        <v>36</v>
+      </c>
+      <c r="I3" t="s">
         <v>37</v>
       </c>
+      <c r="J3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K3" t="s">
+        <v>36</v>
+      </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" t="s">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
         <v>27</v>
       </c>
-      <c r="E3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G3" t="s">
-        <v>50</v>
-      </c>
-      <c r="H3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I3" t="s">
-        <v>38</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="C4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" t="s">
         <v>39</v>
       </c>
-      <c r="K3" t="s">
-        <v>37</v>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" t="s">
+        <v>36</v>
+      </c>
+      <c r="K4" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F4" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>30</v>
       </c>
-      <c r="H4" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4" t="s">
-        <v>37</v>
-      </c>
-      <c r="J4" t="s">
-        <v>37</v>
-      </c>
-      <c r="K4" t="s">
-        <v>37</v>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" t="s">
-        <v>35</v>
-      </c>
-      <c r="H5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I5" t="s">
-        <v>37</v>
-      </c>
-      <c r="J5" t="s">
-        <v>37</v>
-      </c>
-      <c r="K5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
@@ -728,7 +728,7 @@
         <v>9</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F6">
         <v>2022</v>
@@ -740,53 +740,53 @@
         <v>10</v>
       </c>
       <c r="I6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" t="s">
         <v>41</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>43</v>
-      </c>
-      <c r="D7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" t="s">
-        <v>44</v>
       </c>
       <c r="F7">
         <v>2024</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
         <v>11</v>
@@ -810,13 +810,13 @@
         <v>14</v>
       </c>
       <c r="I8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>